<commit_message>
docs(pendientes): agrega MS Schippers - 6 productos sin foto, 45/45 imagenes OK
</commit_message>
<xml_diff>
--- a/docs/PENDIENTES-FOTOS.xlsx
+++ b/docs/PENDIENTES-FOTOS.xlsx
@@ -298,8 +298,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblPendientes" displayName="tblPendientes" ref="A1:H19" headerRowCount="1">
-  <autoFilter ref="A1:H19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblPendientes" displayName="tblPendientes" ref="A1:H25" headerRowCount="1">
+  <autoFilter ref="A1:H25"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Marca"/>
     <tableColumn id="2" name="Código"/>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1398,8 +1398,260 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>3409680</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>(sin foto)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Sorting paddle red, 102 cm</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>🔄 pedir foto real</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Pedir foto real a almacén.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>809599</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>(sin foto)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>High pressure spray gun ST-2600, KEW (blue)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>No tiene foto propia. El código 809660 (misma pistola ST-2600) usa spray-gun-st2600.jpg, pero es la variante de color distinta; no se asignó para no mostrar un producto diferente.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>🔄 pedir foto real</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar si la foto de 809660 sirve para la versión blue o pedir la foto real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>MS PEROFIXER</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>(sin foto)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>PEROFIXER</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>🔄 pedir foto real</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Pedir foto real a almacén.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>(sin foto)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Q5 G10 1LT CAUTERNARIO DE AMONIO</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>No tiene foto propia. Existe q5-20.png para el Q5 G10 de 20 L (código Q5-20), que es otra presentación; no se asignó para no confundir envases.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>🔄 pedir foto real</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Pedir foto del envase de 1 L a almacén.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>200075552</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>(sin foto)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>MS Boquilla de baja presión</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado. Tiene stock (6).</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>🔄 pedir foto real</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Pedir foto real a almacén.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>5070 WALL</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>(sin foto)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>MS Motobomba TopFoam Wall Demo</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Sin foto</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado. Tiene stock (1).</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>🔄 pedir foto real</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Pedir foto real a almacén.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G19">
+  <conditionalFormatting sqref="G2:G25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"🔄 pedir foto real"</formula>
     </cfRule>
@@ -1410,7 +1662,7 @@
       <formula>"✅ aclarada correcta"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E19">
+  <conditionalFormatting sqref="E2:E25">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Incorrecta"</formula>
     </cfRule>
@@ -1434,7 +1686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1552,50 +1804,50 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>MS Schippers</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>COUNTIF(tblPendientes[Marca],"MS Schippers")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="11">
-        <f>SUM(B6:B12)</f>
+      <c r="B14" s="11">
+        <f>SUM(B6:B13)</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Por estado</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Registros</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>🔄 pedir foto real</t>
-        </is>
-      </c>
-      <c r="B18" s="9">
-        <f>COUNTIF(tblPendientes[Estado],A18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>⬜ pendiente</t>
         </is>
       </c>
       <c r="B19" s="9">
@@ -1604,9 +1856,9 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>✅ aclarada correcta</t>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>⬜ pendiente</t>
         </is>
       </c>
       <c r="B20" s="9">
@@ -1614,43 +1866,54 @@
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>✅ aclarada correcta</t>
+        </is>
+      </c>
+      <c r="B21" s="9">
+        <f>COUNTIF(tblPendientes[Estado],A21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Cómo usar este archivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>1. Revise con almacén cada fila de la hoja 'Pendientes' (filtre por Marca o Estado).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>2. Al resolver una foto, cambie el Estado a '✅ aclarada correcta' (se pone verde solo).</t>
+          <t>1. Revise con almacén cada fila de la hoja 'Pendientes' (filtre por Marca o Estado).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>3. Si almacén proporciona la foto real, reemplácela en public/images/catalogo/&lt;marca&gt;/ y actualice el estado.</t>
+          <t>2. Al resolver una foto, cambie el Estado a '✅ aclarada correcta' (se pone verde solo).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>4. Las filas Tipo='Incorrecta' (rojo) son las prioritarias: la foto muestra otra cosa.</t>
+          <t>3. Si almacén proporciona la foto real, reemplácela en public/images/catalogo/&lt;marca&gt;/ y actualice el estado.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>4. Las filas Tipo='Incorrecta' (rojo) son las prioritarias: la foto muestra otra cosa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>5. Este archivo se regenera desde el acumulado de la sesión; conserve sus cambios de estado en esta copia.</t>
         </is>

</xml_diff>

<commit_message>
feat(schippers): 809599 y Q5 usan foto de variante (pendiente de revision)
</commit_message>
<xml_diff>
--- a/docs/PENDIENTES-FOTOS.xlsx
+++ b/docs/PENDIENTES-FOTOS.xlsx
@@ -1453,7 +1453,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>(sin foto)</t>
+          <t>spray-gun-st2600.jpg</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1463,22 +1463,22 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Sin foto</t>
+          <t>Dudosa</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>No tiene foto propia. El código 809660 (misma pistola ST-2600) usa spray-gun-st2600.jpg, pero es la variante de color distinta; no se asignó para no mostrar un producto diferente.</t>
+          <t>Se asignó la foto de la 809660 (misma pistola ST-2600, variante de otro color) a petición del usuario, pendiente de revisión.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>🔄 pedir foto real</t>
+          <t>⬜ pendiente</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Confirmar si la foto de 809660 sirve para la versión blue o pedir la foto real.</t>
+          <t>Confirmar que la foto sirve para la versión blue o pedir la foto real.</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>(sin foto)</t>
+          <t>q5-20.png</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1547,22 +1547,22 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Sin foto</t>
+          <t>Dudosa</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>No tiene foto propia. Existe q5-20.png para el Q5 G10 de 20 L (código Q5-20), que es otra presentación; no se asignó para no confundir envases.</t>
+          <t>Se asignó la foto del Q5 de 20 L (código Q5-20) a petición del usuario; es otra presentación del mismo producto. Pendiente de revisión.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>🔄 pedir foto real</t>
+          <t>⬜ pendiente</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Pedir foto del envase de 1 L a almacén.</t>
+          <t>Confirmar que la foto del envase de 20 L sirve para el de 1 L o pedir la foto real.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(schippers): elimina producto 809599 del catalogo publico
</commit_message>
<xml_diff>
--- a/docs/PENDIENTES-FOTOS.xlsx
+++ b/docs/PENDIENTES-FOTOS.xlsx
@@ -298,8 +298,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblPendientes" displayName="tblPendientes" ref="A1:H25" headerRowCount="1">
-  <autoFilter ref="A1:H25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblPendientes" displayName="tblPendientes" ref="A1:H24" headerRowCount="1">
+  <autoFilter ref="A1:H24"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Marca"/>
     <tableColumn id="2" name="Código"/>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1448,37 +1448,37 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>809599</t>
+          <t>MS PEROFIXER</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>spray-gun-st2600.jpg</t>
+          <t>(sin foto)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>High pressure spray gun ST-2600, KEW (blue)</t>
+          <t>PEROFIXER</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Dudosa</t>
+          <t>Sin foto</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Se asignó la foto de la 809660 (misma pistola ST-2600, variante de otro color) a petición del usuario, pendiente de revisión.</t>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>⬜ pendiente</t>
+          <t>🔄 pedir foto real</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Confirmar que la foto sirve para la versión blue o pedir la foto real.</t>
+          <t>Pedir foto real a almacén.</t>
         </is>
       </c>
     </row>
@@ -1490,37 +1490,37 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>MS PEROFIXER</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>(sin foto)</t>
+          <t>q5-20.png</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>PEROFIXER</t>
+          <t>Q5 G10 1LT CAUTERNARIO DE AMONIO</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Sin foto</t>
+          <t>Dudosa</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado.</t>
+          <t>Se asignó la foto del Q5 de 20 L (código Q5-20) a petición del usuario; es otra presentación del mismo producto. Pendiente de revisión.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>🔄 pedir foto real</t>
+          <t>⬜ pendiente</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Pedir foto real a almacén.</t>
+          <t>Confirmar que la foto del envase de 20 L sirve para el de 1 L o pedir la foto real.</t>
         </is>
       </c>
     </row>
@@ -1532,37 +1532,37 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>200075552</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>q5-20.png</t>
+          <t>(sin foto)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Q5 G10 1LT CAUTERNARIO DE AMONIO</t>
+          <t>MS Boquilla de baja presión</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Dudosa</t>
+          <t>Sin foto</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Se asignó la foto del Q5 de 20 L (código Q5-20) a petición del usuario; es otra presentación del mismo producto. Pendiente de revisión.</t>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado. Tiene stock (6).</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>⬜ pendiente</t>
+          <t>🔄 pedir foto real</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Confirmar que la foto del envase de 20 L sirve para el de 1 L o pedir la foto real.</t>
+          <t>Pedir foto real a almacén.</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>200075552</t>
+          <t>5070 WALL</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>MS Boquilla de baja presión</t>
+          <t>MS Motobomba TopFoam Wall Demo</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado. Tiene stock (6).</t>
+          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado. Tiene stock (1).</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1608,50 +1608,8 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>MS Schippers</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>5070 WALL</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>(sin foto)</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>MS Motobomba TopFoam Wall Demo</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Sin foto</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>El producto no tiene imagen asignada; no existe archivo en disco ni en el catálogo autorizado. Tiene stock (1).</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>🔄 pedir foto real</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Pedir foto real a almacén.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G25">
+  <conditionalFormatting sqref="G2:G24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"🔄 pedir foto real"</formula>
     </cfRule>
@@ -1662,7 +1620,7 @@
       <formula>"✅ aclarada correcta"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E25">
+  <conditionalFormatting sqref="E2:E24">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Incorrecta"</formula>
     </cfRule>

</xml_diff>